<commit_message>
feat: mcp server voor codelijst beheer
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
@@ -529,7 +529,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Collection</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D2" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_92</v>
@@ -651,7 +651,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Collection</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D3" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1096|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_2217</v>
@@ -1535,7 +1535,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/grondwater</v>
       </c>
       <c r="M10" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N10" t="str">
         <v>null</v>
@@ -1657,7 +1657,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/oppervlaktewater</v>
       </c>
       <c r="M11" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N11" t="str">
         <v>null</v>
@@ -1779,7 +1779,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/riool</v>
       </c>
       <c r="M12" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N12" t="str">
         <v>null</v>
@@ -1871,7 +1871,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D13" t="str">
         <v>null</v>
@@ -2023,7 +2023,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/lozingspunt-lozingsplaats</v>
       </c>
       <c r="M14" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N14" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -2145,7 +2145,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-diameter</v>
       </c>
       <c r="M15" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N15" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -2267,7 +2267,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-hoogte</v>
       </c>
       <c r="M16" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N16" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -2389,7 +2389,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt</v>
       </c>
       <c r="M17" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N17" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -2511,7 +2511,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/fakkel</v>
       </c>
       <c r="M18" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N18" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -2633,7 +2633,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/gebouw</v>
       </c>
       <c r="M19" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N19" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -2755,7 +2755,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt</v>
       </c>
       <c r="M20" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N20" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -2877,7 +2877,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="M21" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N21" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -2999,7 +2999,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom</v>
       </c>
       <c r="M22" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N22" t="str">
         <v>null</v>
@@ -3121,7 +3121,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_verticale_uitstroom</v>
       </c>
       <c r="M23" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N23" t="str">
         <v>null</v>
@@ -3213,7 +3213,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D24" t="str">
         <v>null</v>
@@ -3335,7 +3335,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D25" t="str">
         <v>null</v>
@@ -3457,7 +3457,7 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D26" t="str">
         <v>null</v>
@@ -3609,7 +3609,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/injectie</v>
       </c>
       <c r="M27" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N27" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -3731,7 +3731,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/omkeerbaar</v>
       </c>
       <c r="M28" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N28" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -3853,7 +3853,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/peil</v>
       </c>
       <c r="M29" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N29" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -3975,7 +3975,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/pomp</v>
       </c>
       <c r="M30" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N30" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -4097,7 +4097,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerd_vermogen</v>
       </c>
       <c r="M31" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N31" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4219,7 +4219,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_opslagcapaciteit</v>
       </c>
       <c r="M32" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N32" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4341,7 +4341,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_productiecapaciteit</v>
       </c>
       <c r="M33" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N33" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4463,7 +4463,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/luchtzuiverings_techniek</v>
       </c>
       <c r="M34" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N34" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4585,7 +4585,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_energie_productie</v>
       </c>
       <c r="M35" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N35" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4707,7 +4707,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement</v>
       </c>
       <c r="M36" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N36" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -4829,7 +4829,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_percentage</v>
       </c>
       <c r="M37" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N37" t="str">
         <v>null</v>
@@ -4951,7 +4951,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_stof</v>
       </c>
       <c r="M38" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N38" t="str">
         <v>null</v>
@@ -5073,7 +5073,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek</v>
       </c>
       <c r="M39" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -5195,7 +5195,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_ingebruikvan</v>
       </c>
       <c r="M40" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N40" t="str">
         <v>null</v>
@@ -5317,7 +5317,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_techniek</v>
       </c>
       <c r="M41" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N41" t="str">
         <v>null</v>
@@ -5439,7 +5439,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="M42" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N42" t="str">
         <v>null</v>
@@ -5561,7 +5561,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/geothermisch</v>
       </c>
       <c r="M43" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N43" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -5683,7 +5683,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/gpbv</v>
       </c>
       <c r="M44" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N44" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -5805,7 +5805,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/installatie</v>
       </c>
       <c r="M45" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N45" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -5927,7 +5927,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/luchtzuivering</v>
       </c>
       <c r="M46" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N46" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -6049,7 +6049,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/opslag_overslag</v>
       </c>
       <c r="M47" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N47" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -6171,7 +6171,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
       </c>
       <c r="M48" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N48" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -6293,7 +6293,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/waterzuivering</v>
       </c>
       <c r="M49" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N49" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -6415,7 +6415,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/diepte</v>
       </c>
       <c r="M50" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N50" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -6537,7 +6537,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt</v>
       </c>
       <c r="M51" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N51" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -6659,7 +6659,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_diepte</v>
       </c>
       <c r="M52" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N52" t="str">
         <v>null</v>
@@ -6781,7 +6781,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_naam</v>
       </c>
       <c r="M53" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N53" t="str">
         <v>null</v>
@@ -6903,7 +6903,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/controleinrichting</v>
       </c>
       <c r="M54" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N54" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -7025,7 +7025,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/debietmeter</v>
       </c>
       <c r="M55" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N55" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -7147,7 +7147,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/peilput</v>
       </c>
       <c r="M56" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N56" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -7269,7 +7269,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-eigenschappen/diepte</v>
       </c>
       <c r="M57" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N57" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -7391,7 +7391,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-eigenschappen/watervoerendelaag</v>
       </c>
       <c r="M58" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N58" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -7513,7 +7513,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/opnamepunt</v>
       </c>
       <c r="M59" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N59" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -7635,7 +7635,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/pompput</v>
       </c>
       <c r="M60" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N60" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -9587,7 +9587,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-be</v>
       </c>
       <c r="M76" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N76" t="str">
         <v>null</v>
@@ -9709,7 +9709,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-be-naam</v>
       </c>
       <c r="M77" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N77" t="str">
         <v>null</v>
@@ -9831,7 +9831,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-be-on</v>
       </c>
       <c r="M78" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N78" t="str">
         <v>null</v>
@@ -9953,7 +9953,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-be-ve</v>
       </c>
       <c r="M79" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N79" t="str">
         <v>null</v>
@@ -10075,7 +10075,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-buitenland</v>
       </c>
       <c r="M80" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N80" t="str">
         <v>null</v>
@@ -10197,7 +10197,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-buitenland-btw</v>
       </c>
       <c r="M81" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N81" t="str">
         <v>null</v>
@@ -10319,7 +10319,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-buitenland-naam</v>
       </c>
       <c r="M82" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N82" t="str">
         <v>null</v>
@@ -10441,7 +10441,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-none</v>
       </c>
       <c r="M83" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N83" t="str">
         <v>null</v>
@@ -10563,7 +10563,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-none-adres</v>
       </c>
       <c r="M84" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N84" t="str">
         <v>null</v>
@@ -10685,7 +10685,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-none-naam</v>
       </c>
       <c r="M85" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N85" t="str">
         <v>null</v>
@@ -10807,7 +10807,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-werf</v>
       </c>
       <c r="M86" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N86" t="str">
         <v>null</v>
@@ -10929,7 +10929,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-werf-naam</v>
       </c>
       <c r="M87" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N87" t="str">
         <v>null</v>
@@ -11173,7 +11173,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof</v>
       </c>
       <c r="M89" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N89" t="str">
         <v>null</v>
@@ -11295,7 +11295,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_bestemming_type</v>
       </c>
       <c r="M90" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N90" t="str">
         <v>null</v>
@@ -11417,7 +11417,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_hoeveelheid</v>
       </c>
       <c r="M91" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N91" t="str">
         <v>null</v>
@@ -11539,7 +11539,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_materiaalcode</v>
       </c>
       <c r="M92" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N92" t="str">
         <v>null</v>
@@ -11661,7 +11661,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_omschrijving</v>
       </c>
       <c r="M93" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N93" t="str">
         <v>null</v>
@@ -11783,7 +11783,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_opmerking</v>
       </c>
       <c r="M94" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N94" t="str">
         <v>null</v>
@@ -11905,7 +11905,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/grondstof_toepassingswijze</v>
       </c>
       <c r="M95" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N95" t="str">
         <v>null</v>
@@ -12027,7 +12027,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/begintoestand</v>
       </c>
       <c r="M96" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N96" t="str">
         <v>null</v>
@@ -12149,7 +12149,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/datum</v>
       </c>
       <c r="M97" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N97" t="str">
         <v>null</v>
@@ -12271,7 +12271,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/diepte</v>
       </c>
       <c r="M98" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N98" t="str">
         <v>null</v>
@@ -12393,7 +12393,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/duur-stil</v>
       </c>
       <c r="M99" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N99" t="str">
         <v>null</v>
@@ -12515,7 +12515,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/eindtoestand</v>
       </c>
       <c r="M100" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N100" t="str">
         <v>null</v>
@@ -12637,7 +12637,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting</v>
       </c>
       <c r="M101" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N101" t="str">
         <v>null</v>
@@ -12759,7 +12759,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-bemonsteringsinstrument</v>
       </c>
       <c r="M102" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N102" t="str">
         <v>null</v>
@@ -12881,7 +12881,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-datum</v>
       </c>
       <c r="M103" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N103" t="str">
         <v>null</v>
@@ -13003,7 +13003,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-diepte</v>
       </c>
       <c r="M104" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N104" t="str">
         <v>null</v>
@@ -13125,7 +13125,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-labo</v>
       </c>
       <c r="M105" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N105" t="str">
         <v>null</v>
@@ -13247,7 +13247,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-labo-naam</v>
       </c>
       <c r="M106" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N106" t="str">
         <v>null</v>
@@ -13369,7 +13369,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-monsternummer</v>
       </c>
       <c r="M107" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N107" t="str">
         <v>null</v>
@@ -13491,7 +13491,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter</v>
       </c>
       <c r="M108" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N108" t="str">
         <v>null</v>
@@ -13613,7 +13613,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter-datum</v>
       </c>
       <c r="M109" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N109" t="str">
         <v>null</v>
@@ -13735,7 +13735,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter-limiet</v>
       </c>
       <c r="M110" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N110" t="str">
         <v>null</v>
@@ -13857,7 +13857,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter-meetwaarde</v>
       </c>
       <c r="M111" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N111" t="str">
         <v>null</v>
@@ -13979,7 +13979,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter-methode</v>
       </c>
       <c r="M112" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N112" t="str">
         <v>null</v>
@@ -14101,7 +14101,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-parameter-parameter</v>
       </c>
       <c r="M113" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N113" t="str">
         <v>null</v>
@@ -14223,7 +14223,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-referentiepunt</v>
       </c>
       <c r="M114" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N114" t="str">
         <v>null</v>
@@ -14345,7 +14345,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting-techniek</v>
       </c>
       <c r="M115" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N115" t="str">
         <v>null</v>
@@ -14467,7 +14467,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/kwaliteitsmeting_feature</v>
       </c>
       <c r="M116" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N116" t="str">
         <v>null</v>
@@ -14589,7 +14589,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/onttrekking</v>
       </c>
       <c r="M117" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N117" t="str">
         <v>null</v>
@@ -14711,7 +14711,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/onttrekking_feature</v>
       </c>
       <c r="M118" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N118" t="str">
         <v>null</v>
@@ -14833,7 +14833,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/peilmethode</v>
       </c>
       <c r="M119" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N119" t="str">
         <v>null</v>
@@ -14955,7 +14955,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/peilmeting</v>
       </c>
       <c r="M120" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N120" t="str">
         <v>null</v>
@@ -15077,7 +15077,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/peilmeting_feature</v>
       </c>
       <c r="M121" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N121" t="str">
         <v>null</v>
@@ -15199,7 +15199,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/periode</v>
       </c>
       <c r="M122" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N122" t="str">
         <v>null</v>
@@ -15321,7 +15321,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/pomptoestand</v>
       </c>
       <c r="M123" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N123" t="str">
         <v>null</v>
@@ -15443,7 +15443,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/referentiepunt</v>
       </c>
       <c r="M124" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N124" t="str">
         <v>null</v>
@@ -15565,7 +15565,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/type-debiet</v>
       </c>
       <c r="M125" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N125" t="str">
         <v>null</v>
@@ -15687,7 +15687,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/volume</v>
       </c>
       <c r="M126" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N126" t="str">
         <v>null</v>
@@ -15809,7 +15809,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/volume-rust</v>
       </c>
       <c r="M127" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N127" t="str">
         <v>null</v>
@@ -15931,7 +15931,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondwater/volume-werking</v>
       </c>
       <c r="M128" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N128" t="str">
         <v>null</v>
@@ -16053,7 +16053,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/afvalproduct</v>
       </c>
       <c r="M129" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N129" t="str">
         <v>null</v>
@@ -16175,7 +16175,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/afvalproduct_aard</v>
       </c>
       <c r="M130" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N130" t="str">
         <v>null</v>
@@ -16297,7 +16297,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/afvalproduct_hoeveelheid</v>
       </c>
       <c r="M131" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N131" t="str">
         <v>null</v>
@@ -16419,7 +16419,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/afvalproduct_naam</v>
       </c>
       <c r="M132" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N132" t="str">
         <v>null</v>
@@ -16541,7 +16541,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/brandstof</v>
       </c>
       <c r="M133" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N133" t="str">
         <v>null</v>
@@ -16663,7 +16663,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/brandstof_as</v>
       </c>
       <c r="M134" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N134" t="str">
         <v>null</v>
@@ -16785,7 +16785,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/brandstof_naam</v>
       </c>
       <c r="M135" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N135" t="str">
         <v>null</v>
@@ -16907,7 +16907,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/brandstof_s</v>
       </c>
       <c r="M136" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N136" t="str">
         <v>null</v>
@@ -17029,7 +17029,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/brandstof_verbruik</v>
       </c>
       <c r="M137" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N137" t="str">
         <v>null</v>
@@ -17151,7 +17151,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie</v>
       </c>
       <c r="M138" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N138" t="str">
         <v>null</v>
@@ -17273,7 +17273,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_luchtoverschot</v>
       </c>
       <c r="M139" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N139" t="str">
         <v>null</v>
@@ -17395,7 +17395,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_parameter</v>
       </c>
       <c r="M140" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N140" t="str">
         <v>null</v>
@@ -17517,7 +17517,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_parameter_massastroom</v>
       </c>
       <c r="M141" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N141" t="str">
         <v>null</v>
@@ -17639,7 +17639,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_parameter_meetfrequentie</v>
       </c>
       <c r="M142" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N142" t="str">
         <v>null</v>
@@ -17761,7 +17761,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_parameter_parameter</v>
       </c>
       <c r="M143" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N143" t="str">
         <v>null</v>
@@ -17883,7 +17883,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_parameter_standaardafwijking</v>
       </c>
       <c r="M144" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N144" t="str">
         <v>null</v>
@@ -18005,7 +18005,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_temperatuur</v>
       </c>
       <c r="M145" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N145" t="str">
         <v>null</v>
@@ -18127,7 +18127,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_vochtgehalte</v>
       </c>
       <c r="M146" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N146" t="str">
         <v>null</v>
@@ -18249,7 +18249,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissie_zuurstofgehalte</v>
       </c>
       <c r="M147" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N147" t="str">
         <v>null</v>
@@ -18371,7 +18371,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissieduur</v>
       </c>
       <c r="M148" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N148" t="str">
         <v>null</v>
@@ -18493,7 +18493,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissieperiode</v>
       </c>
       <c r="M149" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N149" t="str">
         <v>null</v>
@@ -18615,7 +18615,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissieritme</v>
       </c>
       <c r="M150" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N150" t="str">
         <v>null</v>
@@ -18737,7 +18737,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissietoestand</v>
       </c>
       <c r="M151" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N151" t="str">
         <v>null</v>
@@ -18859,7 +18859,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/emissietype</v>
       </c>
       <c r="M152" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N152" t="str">
         <v>null</v>
@@ -19225,7 +19225,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/geproduceerde_stof</v>
       </c>
       <c r="M155" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N155" t="str">
         <v>null</v>
@@ -19347,7 +19347,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/geproduceerde_stof_aard</v>
       </c>
       <c r="M156" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N156" t="str">
         <v>null</v>
@@ -19469,7 +19469,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/geproduceerde_stof_hoeveelheid</v>
       </c>
       <c r="M157" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N157" t="str">
         <v>null</v>
@@ -19591,7 +19591,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/geproduceerde_stof_naam</v>
       </c>
       <c r="M158" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N158" t="str">
         <v>null</v>
@@ -19713,7 +19713,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/verbruikte_stof</v>
       </c>
       <c r="M159" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N159" t="str">
         <v>null</v>
@@ -19835,7 +19835,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/verbruikte_stof_aard</v>
       </c>
       <c r="M160" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N160" t="str">
         <v>null</v>
@@ -19957,7 +19957,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/verbruikte_stof_hoeveelheid</v>
       </c>
       <c r="M161" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N161" t="str">
         <v>null</v>
@@ -20079,7 +20079,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-lucht/verbruikte_stof_naam</v>
       </c>
       <c r="M162" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N162" t="str">
         <v>null</v>
@@ -21421,7 +21421,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-toestand-indicator/droog</v>
       </c>
       <c r="M173" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N173" t="str">
         <v>null</v>
@@ -21543,7 +21543,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-toestand-indicator/nat</v>
       </c>
       <c r="M174" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N174" t="str">
         <v>null</v>
@@ -21665,7 +21665,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/abnormale-lozing</v>
       </c>
       <c r="M175" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N175" t="str">
         <v>null</v>
@@ -21787,7 +21787,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/abnormale-lozing-jaarvracht</v>
       </c>
       <c r="M176" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N176" t="str">
         <v>null</v>
@@ -21909,7 +21909,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/abnormale-lozing-lozingsduur</v>
       </c>
       <c r="M177" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N177" t="str">
         <v>null</v>
@@ -22031,7 +22031,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/abnormale-lozing-stof</v>
       </c>
       <c r="M178" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N178" t="str">
         <v>null</v>
@@ -22153,7 +22153,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/abnormale-lozing-verklaring</v>
       </c>
       <c r="M179" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N179" t="str">
         <v>null</v>
@@ -22397,7 +22397,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing</v>
       </c>
       <c r="M181" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N181" t="str">
         <v>null</v>
@@ -22519,7 +22519,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-bepalingsmethode</v>
       </c>
       <c r="M182" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N182" t="str">
         <v>null</v>
@@ -22641,7 +22641,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-bepalingsmethodeclassificatie</v>
       </c>
       <c r="M183" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N183" t="str">
         <v>null</v>
@@ -22763,7 +22763,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-concentratie</v>
       </c>
       <c r="M184" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N184" t="str">
         <v>null</v>
@@ -22885,7 +22885,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-dagen</v>
       </c>
       <c r="M185" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N185" t="str">
         <v>null</v>
@@ -23007,7 +23007,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-debiet</v>
       </c>
       <c r="M186" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N186" t="str">
         <v>null</v>
@@ -23129,7 +23129,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-jaarvracht</v>
       </c>
       <c r="M187" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N187" t="str">
         <v>null</v>
@@ -23251,7 +23251,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-meetfrequentie</v>
       </c>
       <c r="M188" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N188" t="str">
         <v>null</v>
@@ -23373,7 +23373,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-water/lozing-stof</v>
       </c>
       <c r="M189" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N189" t="str">
         <v>null</v>
@@ -23495,7 +23495,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/datum</v>
       </c>
       <c r="M190" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N190" t="str">
         <v>null</v>
@@ -23739,7 +23739,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/labo</v>
       </c>
       <c r="M192" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N192" t="str">
         <v>null</v>
@@ -23861,7 +23861,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/labo-id</v>
       </c>
       <c r="M193" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N193" t="str">
         <v>null</v>
@@ -23983,7 +23983,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/labo-naam</v>
       </c>
       <c r="M194" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N194" t="str">
         <v>null</v>
@@ -24105,7 +24105,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/meting</v>
       </c>
       <c r="M195" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N195" t="str">
         <v>null</v>
@@ -24227,7 +24227,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter</v>
       </c>
       <c r="M196" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N196" t="str">
         <v>null</v>
@@ -24349,7 +24349,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter-concentratie</v>
       </c>
       <c r="M197" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N197" t="str">
         <v>null</v>
@@ -24471,7 +24471,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter-meetfrequentie</v>
       </c>
       <c r="M198" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N198" t="str">
         <v>null</v>
@@ -24593,7 +24593,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter-meetonzekerheid</v>
       </c>
       <c r="M199" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N199" t="str">
         <v>null</v>
@@ -24715,7 +24715,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter-parameter</v>
       </c>
       <c r="M200" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N200" t="str">
         <v>null</v>
@@ -24837,7 +24837,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-lucht/parameter-soort</v>
       </c>
       <c r="M201" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N201" t="str">
         <v>null</v>
@@ -24959,7 +24959,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/datum</v>
       </c>
       <c r="M202" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N202" t="str">
         <v>null</v>
@@ -25203,7 +25203,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/labo</v>
       </c>
       <c r="M204" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N204" t="str">
         <v>null</v>
@@ -25325,7 +25325,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/labo-id</v>
       </c>
       <c r="M205" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N205" t="str">
         <v>null</v>
@@ -25447,7 +25447,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/labo-naam</v>
       </c>
       <c r="M206" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N206" t="str">
         <v>null</v>
@@ -25569,7 +25569,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/meting</v>
       </c>
       <c r="M207" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N207" t="str">
         <v>null</v>
@@ -25691,7 +25691,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter</v>
       </c>
       <c r="M208" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N208" t="str">
         <v>null</v>
@@ -25813,7 +25813,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter-concentratie</v>
       </c>
       <c r="M209" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N209" t="str">
         <v>null</v>
@@ -25935,7 +25935,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter-meetfrequentie</v>
       </c>
       <c r="M210" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N210" t="str">
         <v>null</v>
@@ -26057,7 +26057,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter-meetonzekerheid</v>
       </c>
       <c r="M211" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N211" t="str">
         <v>null</v>
@@ -26179,7 +26179,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter-parameter</v>
       </c>
       <c r="M212" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N212" t="str">
         <v>null</v>
@@ -26301,7 +26301,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-zelfcontrole-water/parameter-soort</v>
       </c>
       <c r="M213" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N213" t="str">
         <v>null</v>
@@ -27399,7 +27399,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst</v>
       </c>
       <c r="M222" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N222" t="str">
         <v>null</v>
@@ -27521,7 +27521,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst</v>
       </c>
       <c r="M223" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N223" t="str">
         <v>null</v>
@@ -27643,7 +27643,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld</v>
       </c>
       <c r="M224" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N224" t="str">
         <v>null</v>
@@ -27765,7 +27765,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst</v>
       </c>
       <c r="M225" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N225" t="str">
         <v>null</v>
@@ -27887,7 +27887,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/verkeerde_registratie</v>
       </c>
       <c r="M226" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N226" t="str">
         <v>null</v>
@@ -28009,7 +28009,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
       </c>
       <c r="M227" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N227" t="str">
         <v>null</v>
@@ -28863,7 +28863,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-type/uitwisselpunt</v>
       </c>
       <c r="M234" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N234" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -29229,7 +29229,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="M237" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N237" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -29443,7 +29443,7 @@
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C239" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D239" t="str">
         <v>null</v>
@@ -29595,7 +29595,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_type</v>
       </c>
       <c r="M240" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N240" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -29717,7 +29717,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
       </c>
       <c r="M241" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N241" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -30083,7 +30083,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_eigenschappen</v>
       </c>
       <c r="M244" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N244" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
@@ -30205,7 +30205,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
       </c>
       <c r="M245" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N245" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -30449,7 +30449,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
       </c>
       <c r="M247" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N247" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
@@ -31059,7 +31059,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_grondstoffen</v>
       </c>
       <c r="M252" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N252" t="str">
         <v>null</v>
@@ -31181,7 +31181,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_grondwater</v>
       </c>
       <c r="M253" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N253" t="str">
         <v>null</v>
@@ -31547,7 +31547,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_lucht_emissie</v>
       </c>
       <c r="M256" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N256" t="str">
         <v>null</v>
@@ -31669,7 +31669,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_lucht_rapportering</v>
       </c>
       <c r="M257" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N257" t="str">
         <v>null</v>
@@ -32279,7 +32279,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_toestand_indicator</v>
       </c>
       <c r="M262" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N262" t="str">
         <v>null</v>
@@ -32523,7 +32523,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_water_lozing</v>
       </c>
       <c r="M264" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N264" t="str">
         <v>null</v>
@@ -32767,7 +32767,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_zelfcontrole_lucht_meting</v>
       </c>
       <c r="M266" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N266" t="str">
         <v>null</v>
@@ -33133,7 +33133,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_zelfcontrole_water_meting</v>
       </c>
       <c r="M269" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="N269" t="str">
         <v>null</v>
@@ -33591,7 +33591,7 @@
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C273" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D273" t="str">
         <v>null</v>
@@ -33713,7 +33713,7 @@
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C274" t="str">
-        <v>2026-10-07T13:39:34.912Z</v>
+        <v>2026-10-14T09:25:40.927Z</v>
       </c>
       <c r="D274" t="str">
         <v>null</v>

</xml_diff>

<commit_message>
fix: poc en fix voor tom
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
@@ -538,7 +538,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/operationeel_parameters_grondwater</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E2" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_246|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_247|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_251|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_321|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_329|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_337</v>
@@ -666,7 +666,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/operationeel_stoffen_lucht</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E3" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1057|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1060|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1685|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1686|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1901|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1919</v>
@@ -794,7 +794,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/operationeel_stoffen_water</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E4" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_231|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_316|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_333|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_351|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_424|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_46</v>
@@ -922,7 +922,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/opslagcapaciteit_eenheden</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E5" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_32|https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_33|https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_41|https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_83</v>
@@ -1050,7 +1050,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/productiecapaciteit_eenheden</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E6" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_15</v>
@@ -1178,7 +1178,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/vermogen_eenheden</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E7" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/eenheid/E_92</v>
@@ -1306,7 +1306,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/collection/rie-iepr/verwijderingsrendement_stoffen</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E8" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_1096|https://data.omgeving.vlaanderen.be/id/concept/csor/variabele/V_2217</v>
@@ -2202,7 +2202,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/abnormale</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E15" t="str">
         <v>null</v>
@@ -2330,7 +2330,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/geleide</v>
       </c>
       <c r="D16" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E16" t="str">
         <v>null</v>
@@ -2458,7 +2458,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/niet-geleide</v>
       </c>
       <c r="D17" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E17" t="str">
         <v>null</v>
@@ -2586,7 +2586,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/niet-geleide-fakkel</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E18" t="str">
         <v>null</v>
@@ -2714,7 +2714,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/niet-geleide-lekverlies</v>
       </c>
       <c r="D19" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E19" t="str">
         <v>null</v>
@@ -2842,7 +2842,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/niet-geleide-opslagverlies</v>
       </c>
       <c r="D20" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E20" t="str">
         <v>null</v>
@@ -2970,7 +2970,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissie-type/niet-geleide-overslagverlies</v>
       </c>
       <c r="D21" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E21" t="str">
         <v>null</v>
@@ -3098,7 +3098,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/collector</v>
       </c>
       <c r="D22" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E22" t="str">
         <v>null</v>
@@ -3226,7 +3226,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/externe_waterzuivering</v>
       </c>
       <c r="D23" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E23" t="str">
         <v>null</v>
@@ -3610,7 +3610,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen-selectiemogelijkheden/regenwaterriool</v>
       </c>
       <c r="D26" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E26" t="str">
         <v>null</v>
@@ -3866,7 +3866,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/aantal_punten</v>
       </c>
       <c r="D28" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E28" t="str">
         <v>null</v>
@@ -3994,7 +3994,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/diameter</v>
       </c>
       <c r="D29" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E29" t="str">
         <v>null</v>
@@ -4122,7 +4122,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/hoogte</v>
       </c>
       <c r="D30" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E30" t="str">
         <v>null</v>
@@ -4378,7 +4378,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt_lucht</v>
       </c>
       <c r="D32" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E32" t="str">
         <v>null</v>
@@ -4503,10 +4503,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/fakkel</v>
       </c>
       <c r="D33" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E33" t="str">
         <v>null</v>
@@ -4554,7 +4554,7 @@
         <v>null</v>
       </c>
       <c r="T33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U33" t="str">
         <v>null</v>
@@ -4631,10 +4631,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/gebouw</v>
       </c>
       <c r="D34" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E34" t="str">
         <v>null</v>
@@ -4682,7 +4682,7 @@
         <v>null</v>
       </c>
       <c r="T34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U34" t="str">
         <v>null</v>
@@ -4762,7 +4762,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/installatie</v>
       </c>
       <c r="D35" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E35" t="str">
         <v>null</v>
@@ -4810,7 +4810,7 @@
         <v>null</v>
       </c>
       <c r="T35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U35" t="str">
         <v>null</v>
@@ -5018,7 +5018,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="D37" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E37" t="str">
         <v>null</v>
@@ -5066,7 +5066,7 @@
         <v>null</v>
       </c>
       <c r="T37" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U37" t="str">
         <v>null</v>
@@ -5143,10 +5143,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom</v>
       </c>
       <c r="D38" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E38" t="str">
         <v>null</v>
@@ -5194,7 +5194,7 @@
         <v>null</v>
       </c>
       <c r="T38" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U38" t="str">
         <v>null</v>
@@ -5271,10 +5271,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C39" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_verticale_uitstroom</v>
       </c>
       <c r="D39" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E39" t="str">
         <v>null</v>
@@ -5322,7 +5322,7 @@
         <v>null</v>
       </c>
       <c r="T39" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U39" t="str">
         <v>null</v>
@@ -5402,7 +5402,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte</v>
       </c>
       <c r="D40" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E40" t="str">
         <v>null</v>
@@ -5530,7 +5530,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte_pomp</v>
       </c>
       <c r="D41" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E41" t="str">
         <v>null</v>
@@ -5658,7 +5658,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/lengte</v>
       </c>
       <c r="D42" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E42" t="str">
         <v>null</v>
@@ -5786,7 +5786,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/watervoerendeLaag</v>
       </c>
       <c r="D43" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E43" t="str">
         <v>null</v>
@@ -5914,7 +5914,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/filter</v>
       </c>
       <c r="D44" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E44" t="str">
         <v>null</v>
@@ -6039,10 +6039,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/injectie</v>
       </c>
       <c r="D45" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E45" t="str">
         <v>null</v>
@@ -6090,7 +6090,7 @@
         <v>null</v>
       </c>
       <c r="T45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U45" t="str">
         <v>null</v>
@@ -6167,10 +6167,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/omkeerbaar</v>
       </c>
       <c r="D46" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E46" t="str">
         <v>null</v>
@@ -6218,7 +6218,7 @@
         <v>null</v>
       </c>
       <c r="T46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U46" t="str">
         <v>null</v>
@@ -6295,10 +6295,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C47" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/peil</v>
       </c>
       <c r="D47" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E47" t="str">
         <v>null</v>
@@ -6346,7 +6346,7 @@
         <v>null</v>
       </c>
       <c r="T47" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U47" t="str">
         <v>null</v>
@@ -6423,10 +6423,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C48" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/pomp</v>
       </c>
       <c r="D48" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E48" t="str">
         <v>null</v>
@@ -6474,7 +6474,7 @@
         <v>null</v>
       </c>
       <c r="T48" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U48" t="str">
         <v>null</v>
@@ -6554,7 +6554,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/andere</v>
       </c>
       <c r="D49" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E49" t="str">
         <v>null</v>
@@ -6682,7 +6682,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/andere_motor</v>
       </c>
       <c r="D50" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E50" t="str">
         <v>null</v>
@@ -6810,7 +6810,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/andere_stookinstallatie</v>
       </c>
       <c r="D51" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E51" t="str">
         <v>null</v>
@@ -6938,7 +6938,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/boiler</v>
       </c>
       <c r="D52" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E52" t="str">
         <v>null</v>
@@ -7066,7 +7066,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/dieselmotor</v>
       </c>
       <c r="D53" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E53" t="str">
         <v>null</v>
@@ -7194,7 +7194,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/druk</v>
       </c>
       <c r="D54" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E54" t="str">
         <v>null</v>
@@ -7322,7 +7322,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/dual_fuel_motor</v>
       </c>
       <c r="D55" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E55" t="str">
         <v>null</v>
@@ -7450,7 +7450,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/elektriciteit</v>
       </c>
       <c r="D56" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E56" t="str">
         <v>null</v>
@@ -7578,7 +7578,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/gasmotor</v>
       </c>
       <c r="D57" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E57" t="str">
         <v>null</v>
@@ -7706,7 +7706,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/gasturbine</v>
       </c>
       <c r="D58" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E58" t="str">
         <v>null</v>
@@ -7834,7 +7834,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/mechanische_energie</v>
       </c>
       <c r="D59" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E59" t="str">
         <v>null</v>
@@ -7962,7 +7962,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/stoom</v>
       </c>
       <c r="D60" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E60" t="str">
         <v>null</v>
@@ -8090,7 +8090,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/warm_water</v>
       </c>
       <c r="D61" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E61" t="str">
         <v>null</v>
@@ -8218,7 +8218,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/warme_lucht</v>
       </c>
       <c r="D62" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E62" t="str">
         <v>null</v>
@@ -8346,7 +8346,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen-selectiemogelijkheden/wkk</v>
       </c>
       <c r="D63" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E63" t="str">
         <v>null</v>
@@ -8474,7 +8474,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_opslag_overslagcapaciteit</v>
       </c>
       <c r="D64" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E64" t="str">
         <v>null</v>
@@ -8730,7 +8730,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geproduceerde_stof_of_product</v>
       </c>
       <c r="D66" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E66" t="str">
         <v>null</v>
@@ -8986,7 +8986,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/nominaal_thermisch_vermogen</v>
       </c>
       <c r="D68" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E68" t="str">
         <v>null</v>
@@ -9114,7 +9114,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/omschrijving</v>
       </c>
       <c r="D69" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E69" t="str">
         <v>null</v>
@@ -9242,7 +9242,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/opslagen_overgeslagen_stof</v>
       </c>
       <c r="D70" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E70" t="str">
         <v>null</v>
@@ -9370,7 +9370,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/soort_opgewekte_energie</v>
       </c>
       <c r="D71" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E71" t="str">
         <v>null</v>
@@ -9498,7 +9498,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/technische_kenmerken</v>
       </c>
       <c r="D72" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E72" t="str">
         <v>null</v>
@@ -9626,7 +9626,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_opslag_overslag</v>
       </c>
       <c r="D73" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E73" t="str">
         <v>null</v>
@@ -9754,7 +9754,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_stookinstallatie</v>
       </c>
       <c r="D74" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E74" t="str">
         <v>null</v>
@@ -10007,10 +10007,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C76" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_percentage</v>
       </c>
       <c r="D76" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E76" t="str">
         <v>null</v>
@@ -10058,7 +10058,7 @@
         <v>null</v>
       </c>
       <c r="T76" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U76" t="str">
         <v>false</v>
@@ -10135,10 +10135,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C77" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_stof</v>
       </c>
       <c r="D77" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E77" t="str">
         <v>null</v>
@@ -10186,7 +10186,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/luchtzuivering</v>
       </c>
       <c r="T77" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U77" t="str">
         <v>false</v>
@@ -10394,7 +10394,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_ingebruikvan</v>
       </c>
       <c r="D79" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E79" t="str">
         <v>null</v>
@@ -10442,7 +10442,7 @@
         <v>null</v>
       </c>
       <c r="T79" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U79" t="str">
         <v>false</v>
@@ -10519,10 +10519,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_techniek</v>
       </c>
       <c r="D80" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E80" t="str">
         <v>null</v>
@@ -10570,7 +10570,7 @@
         <v>null</v>
       </c>
       <c r="T80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U80" t="str">
         <v>false</v>
@@ -10647,10 +10647,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C81" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="D81" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E81" t="str">
         <v>null</v>
@@ -10698,7 +10698,7 @@
         <v>null</v>
       </c>
       <c r="T81" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U81" t="str">
         <v>null</v>
@@ -10778,7 +10778,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/fakkel</v>
       </c>
       <c r="D82" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E82" t="str">
         <v>null</v>
@@ -11162,7 +11162,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/indirecte_stookinstallatie</v>
       </c>
       <c r="D85" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E85" t="str">
         <v>null</v>
@@ -11210,7 +11210,7 @@
         <v>null</v>
       </c>
       <c r="T85" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="U85" t="str">
         <v>null</v>
@@ -11546,7 +11546,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/productie_installatie</v>
       </c>
       <c r="D88" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E88" t="str">
         <v>null</v>
@@ -11930,7 +11930,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/ander_referentiepunt</v>
       </c>
       <c r="D91" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E91" t="str">
         <v>null</v>
@@ -12058,7 +12058,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/bovenkant_beschermbuis</v>
       </c>
       <c r="D92" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E92" t="str">
         <v>null</v>
@@ -12186,7 +12186,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/bovenkant_peilbuis</v>
       </c>
       <c r="D93" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E93" t="str">
         <v>null</v>
@@ -12314,7 +12314,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/bovenkant_straatpot</v>
       </c>
       <c r="D94" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E94" t="str">
         <v>null</v>
@@ -12442,7 +12442,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/maaiveld</v>
       </c>
       <c r="D95" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E95" t="str">
         <v>null</v>
@@ -12570,7 +12570,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen-selectiemogelijkheden/onbekend</v>
       </c>
       <c r="D96" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E96" t="str">
         <v>null</v>
@@ -12826,7 +12826,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/merk</v>
       </c>
       <c r="D98" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E98" t="str">
         <v>null</v>
@@ -12954,7 +12954,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/putnummer</v>
       </c>
       <c r="D99" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E99" t="str">
         <v>null</v>
@@ -13207,10 +13207,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C101" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_diepte</v>
       </c>
       <c r="D101" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E101" t="str">
         <v>null</v>
@@ -13258,7 +13258,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/peilput</v>
       </c>
       <c r="T101" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U101" t="str">
         <v>false</v>
@@ -13335,10 +13335,10 @@
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C102" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_naam</v>
       </c>
       <c r="D102" t="str">
-        <v>null</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E102" t="str">
         <v>null</v>
@@ -13386,7 +13386,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/peilput</v>
       </c>
       <c r="T102" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="U102" t="str">
         <v>false</v>
@@ -13466,7 +13466,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/serienummer</v>
       </c>
       <c r="D103" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E103" t="str">
         <v>null</v>
@@ -13978,7 +13978,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-eigenschappen/omschrijving</v>
       </c>
       <c r="D107" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E107" t="str">
         <v>null</v>
@@ -15642,7 +15642,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/activiteit</v>
       </c>
       <c r="D120" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E120" t="str">
         <v>null</v>
@@ -15770,7 +15770,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/energieverbruik</v>
       </c>
       <c r="D121" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E121" t="str">
         <v>null</v>
@@ -15898,7 +15898,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/feature</v>
       </c>
       <c r="D122" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E122" t="str">
         <v>null</v>
@@ -16026,7 +16026,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/grondstoffenverbruik</v>
       </c>
       <c r="D123" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E123" t="str">
         <v>null</v>
@@ -16154,7 +16154,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/productievolume</v>
       </c>
       <c r="D124" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E124" t="str">
         <v>null</v>
@@ -16282,7 +16282,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-contextueel/waterverbruik</v>
       </c>
       <c r="D125" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E125" t="str">
         <v>null</v>
@@ -16922,7 +16922,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-be</v>
       </c>
       <c r="D130" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E130" t="str">
         <v>null</v>
@@ -17434,7 +17434,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-buitenland</v>
       </c>
       <c r="D134" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E134" t="str">
         <v>null</v>
@@ -17818,7 +17818,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-none</v>
       </c>
       <c r="D137" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E137" t="str">
         <v>null</v>
@@ -18202,7 +18202,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/operationeel-grondstoffen/bestemmingsidentificatie-werf</v>
       </c>
       <c r="D140" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E140" t="str">
         <v>null</v>
@@ -37146,7 +37146,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-eigenschappen/diepte</v>
       </c>
       <c r="D288" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E288" t="str">
         <v>null</v>
@@ -37274,7 +37274,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-type/pompput</v>
       </c>
       <c r="D289" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E289" t="str">
         <v>null</v>
@@ -37658,7 +37658,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissie_type</v>
       </c>
       <c r="D292" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E292" t="str">
         <v>null</v>
@@ -38042,7 +38042,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_eigenschappen</v>
       </c>
       <c r="D295" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E295" t="str">
         <v>null</v>
@@ -38426,7 +38426,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_soort_opgewekte_energie</v>
       </c>
       <c r="D298" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E298" t="str">
         <v>null</v>
@@ -38682,7 +38682,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type_stookinstallatie</v>
       </c>
       <c r="D300" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E300" t="str">
         <v>null</v>
@@ -39066,7 +39066,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_referentiepunt_naam</v>
       </c>
       <c r="D303" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E303" t="str">
         <v>null</v>
@@ -39962,7 +39962,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_contextueel</v>
       </c>
       <c r="D310" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E310" t="str">
         <v>null</v>
@@ -40090,7 +40090,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_contextueel_iepr</v>
       </c>
       <c r="D311" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E311" t="str">
         <v>null</v>
@@ -40218,7 +40218,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/operationeel_contextueel_iepr_activiteit</v>
       </c>
       <c r="D312" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E312" t="str">
         <v>null</v>
@@ -43162,7 +43162,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_eigenschappen</v>
       </c>
       <c r="D335" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E335" t="str">
         <v>null</v>
@@ -43276,7 +43276,7 @@
         <v>null</v>
       </c>
       <c r="AP335" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/aantal_punten|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/diameter|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/hoogte|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/lozingspunt-lozingsplaats|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte_pomp|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/lengte|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/watervoerendeLaag|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_opslag_overslagcapaciteit|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_productiecapaciteit|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geproduceerde_stof_of_product|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/luchtzuiverings_techniek|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/nominaal_thermisch_vermogen|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/omschrijving|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/opslagen_overgeslagen_stof|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/soort_opgewekte_energie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/technische_kenmerken|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_opslag_overslag|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/merk|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/putnummer|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/serienummer|https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-eigenschappen/omschrijving|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/uitwisselpunt_eigenschappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/aantal_punten|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/diameter|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/hoogte|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/lozingspunt-lozingsplaats|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/diepte_pomp|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/lengte|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-eigenschappen/watervoerendeLaag|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_opslag_overslagcapaciteit|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerde_productiecapaciteit|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geproduceerde_stof_of_product|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/luchtzuiverings_techniek|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/nominaal_thermisch_vermogen|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/omschrijving|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/opslagen_overgeslagen_stof|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/soort_opgewekte_energie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/technische_kenmerken|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_opslag_overslag|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/type_stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_percentage|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement_stof|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_ingebruikvan|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/waterzuiveringstechniek_techniek|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/merk|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/putnummer|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_diepte|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/referentiepunt_naam|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-eigenschappen/serienummer|https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-eigenschappen/omschrijving|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_eigenschappen|https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-eigenschappen/diepte|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/uitwisselpunt_eigenschappen</v>
       </c>
     </row>
     <row r="336">
@@ -43290,7 +43290,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/systeem_type</v>
       </c>
       <c r="D336" t="str">
-        <v>2026-10-20T08:43:32.688Z</v>
+        <v>2026-10-21T11:58:12.462Z</v>
       </c>
       <c r="E336" t="str">
         <v>null</v>
@@ -43404,7 +43404,7 @@
         <v>null</v>
       </c>
       <c r="AP336" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/fakkel|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/opslag_overslag|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt_lucht|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/filter|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/productie_installatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/luchtzuivering|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/waterzuivering|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/geothermisch|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/gpbv|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/peilput|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/debietmeter|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/controleinrichting|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/opnamepunt|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-type/pompput|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/uitwisselpunt_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/fakkel|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/opslag_overslag|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt_lucht|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/fakkel|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/gebouw|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/installatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_verticale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/filter|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/pomp|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/filter_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/injectie|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/omkeerbaar|https://data.omgeving.vlaanderen.be/id/concept/riepr/filter-type/peil|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/productie_installatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/luchtzuivering|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/waterzuivering|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/geothermisch|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/gpbv|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/indirecte_stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/peilput|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/debietmeter|https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/controleinrichting|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/opnamepunt|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type|https://data.omgeving.vlaanderen.be/id/concept/riepr/uitwisselpunt-type/pompput|https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/uitwisselpunt_type</v>
       </c>
     </row>
     <row r="337">

</xml_diff>